<commit_message>
Expand 93A workbook to full search range
</commit_message>
<xml_diff>
--- a/cases/case_260915_report/93A/config.xlsx
+++ b/cases/case_260915_report/93A/config.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fixed_config" sheetId="1" r:id="Ra59562646c364e46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="search_config" sheetId="2" r:id="R63cf934fb7644cf9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channels" sheetId="3" r:id="R3e7f2304d0e441f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="fixed_config" sheetId="1" r:id="R09f38814392941d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="search_config" sheetId="2" r:id="R431acb5cf18c418f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="channels" sheetId="3" r:id="R1b5c9658100c4d35"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -2501,10 +2501,8 @@
       <x:c r="B4" s="7" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C4" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">0</x:t>
-        </x:is>
+      <x:c r="C4" s="7" t="str">
+        <x:v>0:0.02:0.14</x:v>
       </x:c>
       <x:c r="D4" s="7" t="inlineStr">
         <x:is>
@@ -2526,10 +2524,8 @@
       <x:c r="B5" s="7" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C5" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">-0.1,-0.2,-0.3</x:t>
-        </x:is>
+      <x:c r="C5" s="7" t="str">
+        <x:v>-0.34:0.02:0</x:v>
       </x:c>
       <x:c r="D5" s="7" t="inlineStr">
         <x:is>
@@ -2551,10 +2547,8 @@
       <x:c r="B6" s="7" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C6" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">-0.1,0</x:t>
-        </x:is>
+      <x:c r="C6" s="7" t="str">
+        <x:v>-0.2:0.02:0</x:v>
       </x:c>
       <x:c r="D6" s="7" t="inlineStr">
         <x:is>
@@ -2576,10 +2570,8 @@
       <x:c r="B7" s="7" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C7" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">-20:2:0</x:t>
-        </x:is>
+      <x:c r="C7" s="7" t="str">
+        <x:v>-20:1:0</x:v>
       </x:c>
       <x:c r="D7" s="7" t="inlineStr">
         <x:is>
@@ -2601,10 +2593,8 @@
       <x:c r="B8" s="7" t="b">
         <x:v>1</x:v>
       </x:c>
-      <x:c r="C8" s="7" t="inlineStr">
-        <x:is>
-          <x:t xml:space="preserve">-6:2:0</x:t>
-        </x:is>
+      <x:c r="C8" s="7" t="str">
+        <x:v>-6:1:0</x:v>
       </x:c>
       <x:c r="D8" s="7" t="inlineStr">
         <x:is>

</xml_diff>